<commit_message>
Add accordion-toggle, cards-grid, hero blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 60
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-mybeckman-analytical-ultracentrifugation.report.xlsx
+++ b/tools/importer/reports/import-mybeckman-analytical-ultracentrifugation.report.xlsx
@@ -52,7 +52,7 @@
     <t>mybeckman-clinical-trials</t>
   </si>
   <si>
-    <t>2026-10-27T09:24:10.710Z</t>
+    <t>2026-10-28T05:23:15.215Z</t>
   </si>
   <si>
     <t/>
@@ -166,7 +166,7 @@
     <t>mybeckman-leukemia-and-lymphoma</t>
   </si>
   <si>
-    <t>2026-10-27T09:18:33.316Z</t>
+    <t>2026-10-28T05:23:24.250Z</t>
   </si>
   <si>
     <t>https://www.mybeckman.in/resources/disease-research/leukemia-and-lymphoma</t>
@@ -184,7 +184,7 @@
     <t>mybeckman-monoclonal-antibodies</t>
   </si>
   <si>
-    <t>2026-10-27T09:18:40.027Z</t>
+    <t>2026-10-28T05:23:32.803Z</t>
   </si>
   <si>
     <t>https://www.mybeckman.in/resources/disease-research/monoclonal-antibodies</t>
@@ -202,7 +202,7 @@
     <t>mybeckman-biomanufacturing</t>
   </si>
   <si>
-    <t>2026-10-27T09:18:11.479Z</t>
+    <t>2026-10-28T05:22:58.937Z</t>
   </si>
   <si>
     <t>https://www.mybeckman.in/resources/industries/biomanufacturing</t>
@@ -220,7 +220,7 @@
     <t>mybeckman-synthetic-biology</t>
   </si>
   <si>
-    <t>2026-10-27T09:19:02.403Z</t>
+    <t>2026-10-28T05:23:57.178Z</t>
   </si>
   <si>
     <t>https://www.mybeckman.in/resources/industries/synthetic-biology</t>
@@ -238,7 +238,7 @@
     <t>mybeckman-cell-line-development</t>
   </si>
   <si>
-    <t>2026-10-27T09:18:19.043Z</t>
+    <t>2026-10-28T05:23:06.226Z</t>
   </si>
   <si>
     <t>https://www.mybeckman.in/resources/methods/cell-line-development</t>
@@ -256,7 +256,7 @@
     <t>mybeckman-analytical-ultracentrifugation</t>
   </si>
   <si>
-    <t>2026-10-27T09:26:40.893Z</t>
+    <t>2026-10-28T05:38:02.173Z</t>
   </si>
   <si>
     <t>https://www.mybeckman.in/resources/technologies/analytical-ultracentrifugation</t>
@@ -274,7 +274,7 @@
     <t>mybeckman-next-generation-sequencing</t>
   </si>
   <si>
-    <t>2026-10-27T09:18:47.856Z</t>
+    <t>2026-10-28T05:23:40.432Z</t>
   </si>
   <si>
     <t>https://www.mybeckman.in/resources/technologies/next-generation-sequencing</t>
@@ -355,7 +355,7 @@
     <t>mybeckman-protein-production</t>
   </si>
   <si>
-    <t>2026-10-27T09:18:55.176Z</t>
+    <t>2026-10-28T05:23:48.671Z</t>
   </si>
   <si>
     <t>https://www.mybeckman.in/resources/product-applications/process-development-manufacturing/protein-production</t>

</xml_diff>